<commit_message>
rename manufacturer name to manufacturer
</commit_message>
<xml_diff>
--- a/product_upload/packages/1/file.xlsx
+++ b/product_upload/packages/1/file.xlsx
@@ -596,7 +596,7 @@
       </c>
       <c r="AJ1" t="inlineStr">
         <is>
-          <t>Manufacturer Name</t>
+          <t>Manufacturer</t>
         </is>
       </c>
       <c r="AK1" t="inlineStr">
@@ -761,8 +761,10 @@
       <c r="Y2" t="n">
         <v>0</v>
       </c>
-      <c r="Z2" t="n">
-        <v>0</v>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -960,8 +962,10 @@
       <c r="Y3" t="n">
         <v>0</v>
       </c>
-      <c r="Z3" t="n">
-        <v>0</v>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
@@ -1159,8 +1163,10 @@
       <c r="Y4" t="n">
         <v>0</v>
       </c>
-      <c r="Z4" t="n">
-        <v>0</v>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -1362,8 +1368,10 @@
       <c r="Y5" t="n">
         <v>0</v>
       </c>
-      <c r="Z5" t="n">
-        <v>0</v>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -1557,8 +1565,10 @@
       <c r="Y6" t="n">
         <v>0</v>
       </c>
-      <c r="Z6" t="n">
-        <v>0</v>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1760,8 +1770,10 @@
       <c r="Y7" t="n">
         <v>0</v>
       </c>
-      <c r="Z7" t="n">
-        <v>0</v>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1969,7 +1981,7 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Manufacturer name</t>
+          <t>Manufacturer</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
@@ -3536,7 +3548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3617,40 +3629,45 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Size unit</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>Manufacturer *</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Period After Opening.1</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Usage Instructions</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Warnings</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Manufacturer Name</t>
-        </is>
-      </c>
       <c r="V1" t="inlineStr">
         <is>
+          <t>Manufacturer</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>Ingredients</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Seller SKU</t>
         </is>
@@ -3730,38 +3747,43 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>172.2</v>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>SKU-0EA541E6A9B8</t>
         </is>
@@ -3841,38 +3863,43 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>175.42</v>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>SKU-32D5B744278B</t>
         </is>
@@ -3952,38 +3979,43 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>146.59</v>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>SKU-E258203AD54E</t>
         </is>
@@ -4063,38 +4095,43 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>255.68</v>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>SKU-CFAB54E74D89</t>
         </is>
@@ -4174,38 +4211,43 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>337.2</v>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>SKU-7D187EA30596</t>
         </is>
@@ -4285,38 +4327,43 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>385.59</v>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>SKU-86A60E7CF348</t>
         </is>
@@ -4396,38 +4443,43 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>158.19</v>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>SKU-469D96FFC962</t>
         </is>
@@ -4507,38 +4559,43 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>232.7</v>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>SKU-DC85067CD61D</t>
         </is>
@@ -4618,38 +4675,43 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>19.64</v>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="X10" t="inlineStr">
         <is>
           <t>SKU-24ACCCB4226F</t>
         </is>
@@ -4729,38 +4791,43 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>72.48</v>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>SKU-D01695E3CD03</t>
         </is>
@@ -4840,38 +4907,43 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>478.35</v>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>SKU-2FECD9A2C528</t>
         </is>
@@ -4951,38 +5023,43 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>494.37</v>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>SKU-7439B33B9DE4</t>
         </is>
@@ -5062,38 +5139,43 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q14" t="n">
+      <c r="R14" t="n">
         <v>122.58</v>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>SKU-744AEF206672</t>
         </is>
@@ -5173,38 +5255,43 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>490.43</v>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>SKU-B359C693F089</t>
         </is>
@@ -5284,38 +5371,43 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>120.12</v>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>SKU-71E66890A830</t>
         </is>
@@ -5395,38 +5487,43 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q17" t="n">
+      <c r="R17" t="n">
         <v>404.26</v>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>SKU-40074E187278</t>
         </is>
@@ -5506,38 +5603,43 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q18" t="n">
+      <c r="R18" t="n">
         <v>100.25</v>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>SKU-957850B8F25E</t>
         </is>
@@ -5617,38 +5719,43 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>433.97</v>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>SKU-E7CDD3C02D27</t>
         </is>
@@ -5728,38 +5835,43 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q20" t="n">
+      <c r="R20" t="n">
         <v>436.14</v>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>SKU-319E5C1223EE</t>
         </is>
@@ -5839,38 +5951,43 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="Q21" t="n">
+      <c r="R21" t="n">
         <v>125.37</v>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>12M</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>Use as directed</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>Keep out of reach of children</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="V21" t="inlineStr">
         <is>
           <t>Yusur Pharma</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>Aqua, Glycerin</t>
         </is>
       </c>
-      <c r="W21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>SKU-5D507DF3425C</t>
         </is>

</xml_diff>